<commit_message>
Vendor csv and recovery created
</commit_message>
<xml_diff>
--- a/vendor-performance/datasets/vendor-corrective-actions.xlsx
+++ b/vendor-performance/datasets/vendor-corrective-actions.xlsx
@@ -1,10 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" mc:Ignorable="x15">
-  <fileVersion appName="xl" lastEdited="6" lowestEdited="6" rupBuild="14420"/>
-  <workbookPr defaultThemeVersion="164011"/>
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="29929"/>
+  <workbookPr/>
+  <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+    <mc:Choice Requires="x15">
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/1e29a6debf5eaf8e/Documents/GitHub/northstar-health-operations/vendor-performance/datasets/"/>
+    </mc:Choice>
+  </mc:AlternateContent>
+  <xr:revisionPtr revIDLastSave="13" documentId="11_F25DC773A252ABDACC104871895B64DE5BDE58EE" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{E4C2FC8C-DDBC-433A-81EB-A50E25B68791}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="0" windowWidth="22260" windowHeight="12645"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="38640" windowHeight="21120" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -18,8 +24,232 @@
 </workbook>
 </file>
 
+<file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="80" uniqueCount="72">
+  <si>
+    <t>corrective_action_id</t>
+  </si>
+  <si>
+    <t>vendor_id</t>
+  </si>
+  <si>
+    <t>corrective_action_type</t>
+  </si>
+  <si>
+    <t>corrective_action_status</t>
+  </si>
+  <si>
+    <t>corrective_action_severity</t>
+  </si>
+  <si>
+    <t>trigger_reason</t>
+  </si>
+  <si>
+    <t>sla_event_id</t>
+  </si>
+  <si>
+    <t>fulfillment_event_id</t>
+  </si>
+  <si>
+    <t>related_ticket_id</t>
+  </si>
+  <si>
+    <t>assigned_owner</t>
+  </si>
+  <si>
+    <t>remediation_plan_summary</t>
+  </si>
+  <si>
+    <t>monitoring_start_date</t>
+  </si>
+  <si>
+    <t>reassessment_date</t>
+  </si>
+  <si>
+    <t>recovery_status</t>
+  </si>
+  <si>
+    <t>escalation_required_flag</t>
+  </si>
+  <si>
+    <t>corrective_action_closed_flag</t>
+  </si>
+  <si>
+    <t>notes</t>
+  </si>
+  <si>
+    <t>CA-1001</t>
+  </si>
+  <si>
+    <t>VEND-003</t>
+  </si>
+  <si>
+    <t>SLA Recovery</t>
+  </si>
+  <si>
+    <t>Monitoring</t>
+  </si>
+  <si>
+    <t>Action Required</t>
+  </si>
+  <si>
+    <t>Repeated SLA breaches triggered operational review.</t>
+  </si>
+  <si>
+    <t>SLA-1002</t>
+  </si>
+  <si>
+    <t>VF-1002</t>
+  </si>
+  <si>
+    <t>INC-100012</t>
+  </si>
+  <si>
+    <t>Vendor Management</t>
+  </si>
+  <si>
+    <t>Vendor required to improve fulfillment response consistency and reduce shipment delays.</t>
+  </si>
+  <si>
+    <t>Improving</t>
+  </si>
+  <si>
+    <t>Vendor escalation activity decreased but monitoring remains active.</t>
+  </si>
+  <si>
+    <t>CA-1002</t>
+  </si>
+  <si>
+    <t>VEND-004</t>
+  </si>
+  <si>
+    <t>Fulfillment Stabilization</t>
+  </si>
+  <si>
+    <t>Escalated Review</t>
+  </si>
+  <si>
+    <t>Delayed and partial fulfillment events created operational disruption exposure.</t>
+  </si>
+  <si>
+    <t>SLA-1006</t>
+  </si>
+  <si>
+    <t>VF-1006</t>
+  </si>
+  <si>
+    <t>INC-100001</t>
+  </si>
+  <si>
+    <t>Supply Chain Operations</t>
+  </si>
+  <si>
+    <t>Vendor required to stabilize shipment completion reliability and improve communication timelines.</t>
+  </si>
+  <si>
+    <t>Unresolved</t>
+  </si>
+  <si>
+    <t>Repeated delayed shipment activity continues during monitoring period.</t>
+  </si>
+  <si>
+    <t>CA-1003</t>
+  </si>
+  <si>
+    <t>VEND-002</t>
+  </si>
+  <si>
+    <t>Operational Recovery</t>
+  </si>
+  <si>
+    <t>Resolved</t>
+  </si>
+  <si>
+    <t>Escalation-linked shipment delays required operational remediation review.</t>
+  </si>
+  <si>
+    <t>SLA-1003</t>
+  </si>
+  <si>
+    <t>VF-1003</t>
+  </si>
+  <si>
+    <t>INC-100007</t>
+  </si>
+  <si>
+    <t>Operational Support</t>
+  </si>
+  <si>
+    <t>Vendor communication expectations reviewed and escalation procedures clarified.</t>
+  </si>
+  <si>
+    <t>Stable</t>
+  </si>
+  <si>
+    <t>Operational escalation frequency decreased after remediation review.</t>
+  </si>
+  <si>
+    <t>CA-1004</t>
+  </si>
+  <si>
+    <t>VEND-005</t>
+  </si>
+  <si>
+    <t>Continuity Risk Review</t>
+  </si>
+  <si>
+    <t>Backup supplier fulfillment delays increased continuity-sensitive monitoring requirements.</t>
+  </si>
+  <si>
+    <t>SLA-1004</t>
+  </si>
+  <si>
+    <t>VF-1004</t>
+  </si>
+  <si>
+    <t>Inventory Leadership</t>
+  </si>
+  <si>
+    <t>Vendor required to improve replenishment timeline transparency during backup supply periods.</t>
+  </si>
+  <si>
+    <t>Vendor performance remains under continuity-risk observation.</t>
+  </si>
+  <si>
+    <t>CA-1005</t>
+  </si>
+  <si>
+    <t>VEND-001</t>
+  </si>
+  <si>
+    <t>Escalation Reduction</t>
+  </si>
+  <si>
+    <t>Advisory</t>
+  </si>
+  <si>
+    <t>Minor escalation review initiated following temporary shipment coordination concerns.</t>
+  </si>
+  <si>
+    <t>SLA-1005</t>
+  </si>
+  <si>
+    <t>VF-1005</t>
+  </si>
+  <si>
+    <t>Vendor coordination processes reviewed with no additional corrective escalation required.</t>
+  </si>
+  <si>
+    <t>Vendor returned to normal operational monitoring status.</t>
+  </si>
+</sst>
+</file>
+
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" mc:Ignorable="x14ac x16r2">
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
+  <numFmts count="1">
+    <numFmt numFmtId="165" formatCode="yyyy\-mm\-dd;@"/>
+  </numFmts>
   <fonts count="1" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
@@ -49,8 +279,9 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="1">
+  <cellXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
+    <xf numFmtId="165" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -330,10 +561,328 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1"/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
+  <dimension ref="A1:Q6"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
-  <sheetData/>
+  <cols>
+    <col min="11" max="11" width="92.28515625" bestFit="1" customWidth="1"/>
+    <col min="12" max="12" width="21.140625" style="1" bestFit="1" customWidth="1"/>
+    <col min="13" max="13" width="31.140625" style="1" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:17" x14ac:dyDescent="0.25">
+      <c r="A1" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" t="s">
+        <v>1</v>
+      </c>
+      <c r="C1" t="s">
+        <v>2</v>
+      </c>
+      <c r="D1" t="s">
+        <v>3</v>
+      </c>
+      <c r="E1" t="s">
+        <v>4</v>
+      </c>
+      <c r="F1" t="s">
+        <v>5</v>
+      </c>
+      <c r="G1" t="s">
+        <v>6</v>
+      </c>
+      <c r="H1" t="s">
+        <v>7</v>
+      </c>
+      <c r="I1" t="s">
+        <v>8</v>
+      </c>
+      <c r="J1" t="s">
+        <v>9</v>
+      </c>
+      <c r="K1" t="s">
+        <v>10</v>
+      </c>
+      <c r="L1" s="1" t="s">
+        <v>11</v>
+      </c>
+      <c r="M1" s="1" t="s">
+        <v>12</v>
+      </c>
+      <c r="N1" t="s">
+        <v>13</v>
+      </c>
+      <c r="O1" t="s">
+        <v>14</v>
+      </c>
+      <c r="P1" t="s">
+        <v>15</v>
+      </c>
+      <c r="Q1" t="s">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="2" spans="1:17" x14ac:dyDescent="0.25">
+      <c r="A2" t="s">
+        <v>17</v>
+      </c>
+      <c r="B2" t="s">
+        <v>18</v>
+      </c>
+      <c r="C2" t="s">
+        <v>19</v>
+      </c>
+      <c r="D2" t="s">
+        <v>20</v>
+      </c>
+      <c r="E2" t="s">
+        <v>21</v>
+      </c>
+      <c r="F2" t="s">
+        <v>22</v>
+      </c>
+      <c r="G2" t="s">
+        <v>23</v>
+      </c>
+      <c r="H2" t="s">
+        <v>24</v>
+      </c>
+      <c r="I2" t="s">
+        <v>25</v>
+      </c>
+      <c r="J2" t="s">
+        <v>26</v>
+      </c>
+      <c r="K2" t="s">
+        <v>27</v>
+      </c>
+      <c r="L2" s="1">
+        <v>46166</v>
+      </c>
+      <c r="M2" s="1">
+        <v>46180</v>
+      </c>
+      <c r="N2" t="s">
+        <v>28</v>
+      </c>
+      <c r="O2" t="b">
+        <v>1</v>
+      </c>
+      <c r="P2" t="b">
+        <v>0</v>
+      </c>
+      <c r="Q2" t="s">
+        <v>29</v>
+      </c>
+    </row>
+    <row r="3" spans="1:17" x14ac:dyDescent="0.25">
+      <c r="A3" t="s">
+        <v>30</v>
+      </c>
+      <c r="B3" t="s">
+        <v>31</v>
+      </c>
+      <c r="C3" t="s">
+        <v>32</v>
+      </c>
+      <c r="D3" t="s">
+        <v>33</v>
+      </c>
+      <c r="E3" t="s">
+        <v>33</v>
+      </c>
+      <c r="F3" t="s">
+        <v>34</v>
+      </c>
+      <c r="G3" t="s">
+        <v>35</v>
+      </c>
+      <c r="H3" t="s">
+        <v>36</v>
+      </c>
+      <c r="I3" t="s">
+        <v>37</v>
+      </c>
+      <c r="J3" t="s">
+        <v>38</v>
+      </c>
+      <c r="K3" t="s">
+        <v>39</v>
+      </c>
+      <c r="L3" s="1">
+        <v>46166</v>
+      </c>
+      <c r="M3" s="1">
+        <v>46183</v>
+      </c>
+      <c r="N3" t="s">
+        <v>40</v>
+      </c>
+      <c r="O3" t="b">
+        <v>1</v>
+      </c>
+      <c r="P3" t="b">
+        <v>0</v>
+      </c>
+      <c r="Q3" t="s">
+        <v>41</v>
+      </c>
+    </row>
+    <row r="4" spans="1:17" x14ac:dyDescent="0.25">
+      <c r="A4" t="s">
+        <v>42</v>
+      </c>
+      <c r="B4" t="s">
+        <v>43</v>
+      </c>
+      <c r="C4" t="s">
+        <v>44</v>
+      </c>
+      <c r="D4" t="s">
+        <v>45</v>
+      </c>
+      <c r="E4" t="s">
+        <v>20</v>
+      </c>
+      <c r="F4" t="s">
+        <v>46</v>
+      </c>
+      <c r="G4" t="s">
+        <v>47</v>
+      </c>
+      <c r="H4" t="s">
+        <v>48</v>
+      </c>
+      <c r="I4" t="s">
+        <v>49</v>
+      </c>
+      <c r="J4" t="s">
+        <v>50</v>
+      </c>
+      <c r="K4" t="s">
+        <v>51</v>
+      </c>
+      <c r="L4" s="1">
+        <v>46165</v>
+      </c>
+      <c r="M4" s="1">
+        <v>46172</v>
+      </c>
+      <c r="N4" t="s">
+        <v>52</v>
+      </c>
+      <c r="O4" t="b">
+        <v>0</v>
+      </c>
+      <c r="P4" t="b">
+        <v>1</v>
+      </c>
+      <c r="Q4" t="s">
+        <v>53</v>
+      </c>
+    </row>
+    <row r="5" spans="1:17" x14ac:dyDescent="0.25">
+      <c r="A5" t="s">
+        <v>54</v>
+      </c>
+      <c r="B5" t="s">
+        <v>55</v>
+      </c>
+      <c r="C5" t="s">
+        <v>56</v>
+      </c>
+      <c r="D5" t="s">
+        <v>20</v>
+      </c>
+      <c r="E5" t="s">
+        <v>20</v>
+      </c>
+      <c r="F5" t="s">
+        <v>57</v>
+      </c>
+      <c r="G5" t="s">
+        <v>58</v>
+      </c>
+      <c r="H5" t="s">
+        <v>59</v>
+      </c>
+      <c r="J5" t="s">
+        <v>60</v>
+      </c>
+      <c r="K5" t="s">
+        <v>61</v>
+      </c>
+      <c r="L5" s="1">
+        <v>46166</v>
+      </c>
+      <c r="M5" s="1">
+        <v>46187</v>
+      </c>
+      <c r="N5" t="s">
+        <v>20</v>
+      </c>
+      <c r="O5" t="b">
+        <v>0</v>
+      </c>
+      <c r="P5" t="b">
+        <v>0</v>
+      </c>
+      <c r="Q5" t="s">
+        <v>62</v>
+      </c>
+    </row>
+    <row r="6" spans="1:17" x14ac:dyDescent="0.25">
+      <c r="A6" t="s">
+        <v>63</v>
+      </c>
+      <c r="B6" t="s">
+        <v>64</v>
+      </c>
+      <c r="C6" t="s">
+        <v>65</v>
+      </c>
+      <c r="D6" t="s">
+        <v>45</v>
+      </c>
+      <c r="E6" t="s">
+        <v>66</v>
+      </c>
+      <c r="F6" t="s">
+        <v>67</v>
+      </c>
+      <c r="G6" t="s">
+        <v>68</v>
+      </c>
+      <c r="H6" t="s">
+        <v>69</v>
+      </c>
+      <c r="J6" t="s">
+        <v>26</v>
+      </c>
+      <c r="K6" t="s">
+        <v>70</v>
+      </c>
+      <c r="L6" s="1">
+        <v>46164</v>
+      </c>
+      <c r="M6" s="1">
+        <v>46169</v>
+      </c>
+      <c r="N6" t="s">
+        <v>52</v>
+      </c>
+      <c r="O6" t="b">
+        <v>0</v>
+      </c>
+      <c r="P6" t="b">
+        <v>1</v>
+      </c>
+      <c r="Q6" t="s">
+        <v>71</v>
+      </c>
+    </row>
+  </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
</xml_diff>